<commit_message>
Added news test cases for some processes and updated Field.xlsx file
CXC Process
Update Dispatcher test case
Process test case
Using mock
</commit_message>
<xml_diff>
--- a/MultiProcessesAssistant/Data/Templates/Fields.xlsx
+++ b/MultiProcessesAssistant/Data/Templates/Fields.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Documents\UiPath\RPA_Projects\MultiprocessesAssistant\Data\Templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Documents\GitHub\BOT_001\RPA_Projects\MultiProcessesAssistant\Data\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47DF972A-C3F8-4374-8E81-496F50DB2EEA}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D967641C-FE1A-4F98-AEE1-BD995737AD11}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="732" windowWidth="13812" windowHeight="10464" xr2:uid="{158EB1B0-016B-43AB-8820-CC2EB498F0C2}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="31176" windowHeight="12456" xr2:uid="{158EB1B0-016B-43AB-8820-CC2EB498F0C2}"/>
   </bookViews>
   <sheets>
     <sheet name="CXC" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="46">
   <si>
     <t>Fields</t>
   </si>
@@ -109,13 +109,73 @@
   </si>
   <si>
     <t>IdBankAccount</t>
+  </si>
+  <si>
+    <t>Descripción</t>
+  </si>
+  <si>
+    <t>Saldo que le deben Neto (con retenciones)</t>
+  </si>
+  <si>
+    <t>Colocar el monto que le dieron de anticipo</t>
+  </si>
+  <si>
+    <t>Nombre del banco al cual se quiere que consignen el dinero</t>
+  </si>
+  <si>
+    <t>Ciudad en la que se generará la CXC (ciudad del creador de la cxc o solicitante)</t>
+  </si>
+  <si>
+    <t>Fecha en la que se generará la CXC</t>
+  </si>
+  <si>
+    <t>Nombre la de empresa a la cual se cobrará</t>
+  </si>
+  <si>
+    <t>Nit de la empresa a la cual se cobrar</t>
+  </si>
+  <si>
+    <t>Nombre de la empresa o persona que presto el servicio/producto a cobrar</t>
+  </si>
+  <si>
+    <t>Tipo de identificación de la empresa o persona que presto el servicio/producto a cobrar</t>
+  </si>
+  <si>
+    <t>Número de identificación de la empresa o persona que presto el servicio/producto a cobrar</t>
+  </si>
+  <si>
+    <t>Ciudad en la empresa o persona que presto el servicio/producto a cobrar con la CXC (ciudad del creador de la cxc o solicitante)</t>
+  </si>
+  <si>
+    <t>Saldo que le deben Bruto (sin retenciones)</t>
+  </si>
+  <si>
+    <t>Tipo de divisa (COP, USD, EUR, etc)</t>
+  </si>
+  <si>
+    <t>Descripción del trabajo o servicio que se presto y será cobrado</t>
+  </si>
+  <si>
+    <t>Número de horas totales emmpleadas en el trabajo o servicio que se presto y será cobrado</t>
+  </si>
+  <si>
+    <t>Fecha en la que se comenzo el trabajo o servicio que se presto y será cobrado (formato dd/MM/yyyy)</t>
+  </si>
+  <si>
+    <t>Fecha en la que se finalizo el trabajo o servicio que se presto y será cobrado (formato dd/MM/yyyy)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tipo de cuenta a consignar </t>
+  </si>
+  <si>
+    <t>Número de la cuenta a consignar</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -127,6 +187,21 @@
       <b/>
       <sz val="11"/>
       <color theme="3"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -146,7 +221,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -154,13 +229,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -475,179 +567,243 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B8F3C59-BBD4-4621-AB40-6F7756773ACF}">
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.5546875" customWidth="1"/>
     <col min="2" max="2" width="16.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="121.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C1" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>22</v>
       </c>
       <c r="B2" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C2" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>16</v>
       </c>
       <c r="B3" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C3" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>24</v>
       </c>
       <c r="B4" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C4" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>1</v>
       </c>
       <c r="B5" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C5" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>2</v>
       </c>
       <c r="B6" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C6" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>3</v>
       </c>
       <c r="B7" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C7" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>4</v>
       </c>
       <c r="B8" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C8" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>5</v>
       </c>
       <c r="B9" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C9" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>6</v>
       </c>
       <c r="B10" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C10" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>7</v>
       </c>
       <c r="B11" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C11" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>8</v>
       </c>
       <c r="B12" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C12" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>9</v>
       </c>
       <c r="B13" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C13" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>15</v>
       </c>
       <c r="B14" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C14" s="3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>10</v>
       </c>
       <c r="B15" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C15" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>11</v>
       </c>
       <c r="B16" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C16" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>12</v>
       </c>
       <c r="B17" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C17" s="3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>13</v>
       </c>
       <c r="B18" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C18" s="3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>14</v>
       </c>
       <c r="B19" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C19" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>23</v>
       </c>
       <c r="B20" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C20" s="3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>25</v>
       </c>
       <c r="B21" t="s">
         <v>17</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>